<commit_message>
update ozon ff boxes 2026-07-04
</commit_message>
<xml_diff>
--- a/supplies/108441550-1.xlsx
+++ b/supplies/108441550-1.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инфо" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ПО КОРОБАМ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ПО ТОВАРУ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Инфо" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ПО КОРОБАМ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ПО ТОВАРУ" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
update ozon ff boxes 2026-08-01
</commit_message>
<xml_diff>
--- a/supplies/108441550-1.xlsx
+++ b/supplies/108441550-1.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Витамины для щенков и растущих собак 100 таблеток</t>
+          <t>Витамины для щенков и растущих собак 8in1 Excel Multi Vit Puppy 100 шт</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Витамины для собак мелких пород 70 таблеток</t>
+          <t>Витамины для собак мелких пород Excel Multi Vitamin Small Breed 70 шт</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -719,7 +719,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Витамины для собак крупных пород 80 таблеток</t>
+          <t>Витамины для собак крупных пород 8in1 Excel Brewer's Yeast for large breed 80 шт</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -755,7 +755,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Витамины для собак Glucosamine для суставов 55 таблеток</t>
+          <t>Витамины для собак для суставов 8in1 Excel Glucosamine 55 шт</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -791,7 +791,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Витамины для щенков и растущих собак 100 таблеток</t>
+          <t>Витамины для щенков и растущих собак 8in1 Excel Multi Vit Puppy 100 шт</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -827,7 +827,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Витамины для собак мелких пород 70 таблеток</t>
+          <t>Витамины для собак мелких пород Excel Multi Vitamin Small Breed 70 шт</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -863,7 +863,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Витамины для собак крупных пород 80 таблеток</t>
+          <t>Витамины для собак крупных пород 8in1 Excel Brewer's Yeast for large breed 80 шт</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -899,7 +899,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Витамины для пожилых собак от 5 лет 70 таблеток</t>
+          <t>Витамины для пожилых собак от 5 лет 8in1 Excel Multi Vitamin Senior 70 шт</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -935,7 +935,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Витамины для собак мелких пород 70 таблеток</t>
+          <t>Витамины для собак мелких пород Excel Multi Vitamin Small Breed 70 шт</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -971,7 +971,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Витамины для собак крупных пород 80 таблеток</t>
+          <t>Витамины для собак крупных пород 8in1 Excel Brewer's Yeast for large breed 80 шт</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Витамины для собак Glucosamine для суставов 55 таблеток</t>
+          <t>Витамины для собак для суставов 8in1 Excel Glucosamine 55 шт</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Витамины для щенков и растущих собак 100 таблеток</t>
+          <t>Витамины для щенков и растущих собак 8in1 Excel Multi Vit Puppy 100 шт</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Витамины для собак мелких пород 70 таблеток</t>
+          <t>Витамины для собак мелких пород Excel Multi Vitamin Small Breed 70 шт</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Витамины для собак крупных пород 80 таблеток</t>
+          <t>Витамины для собак крупных пород 8in1 Excel Brewer's Yeast for large breed 80 шт</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Витамины для пожилых собак от 5 лет 70 таблеток</t>
+          <t>Витамины для пожилых собак от 5 лет 8in1 Excel Multi Vitamin Senior 70 шт</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Витамины для собак Glucosamine для суставов 55 таблеток</t>
+          <t>Витамины для собак для суставов 8in1 Excel Glucosamine 55 шт</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Витамины для собак мелких пород 70 таблеток</t>
+          <t>Витамины для собак мелких пород Excel Multi Vitamin Small Breed 70 шт</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Витамины для собак Glucosamine для суставов 55 таблеток</t>
+          <t>Витамины для собак для суставов 8in1 Excel Glucosamine 55 шт</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Витамины для щенков и растущих собак 100 таблеток</t>
+          <t>Витамины для щенков и растущих собак 8in1 Excel Multi Vit Puppy 100 шт</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Витамины для щенков и растущих собак 100 таблеток</t>
+          <t>Витамины для щенков и растущих собак 8in1 Excel Multi Vit Puppy 100 шт</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Витамины для щенков и растущих собак 100 таблеток</t>
+          <t>Витамины для щенков и растущих собак 8in1 Excel Multi Vit Puppy 100 шт</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Витамины для собак крупных пород 80 таблеток</t>
+          <t>Витамины для собак крупных пород 8in1 Excel Brewer's Yeast for large breed 80 шт</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Витамины для собак крупных пород 80 таблеток</t>
+          <t>Витамины для собак крупных пород 8in1 Excel Brewer's Yeast for large breed 80 шт</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Витамины для собак крупных пород 80 таблеток</t>
+          <t>Витамины для собак крупных пород 8in1 Excel Brewer's Yeast for large breed 80 шт</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Витамины для собак крупных пород 80 таблеток</t>
+          <t>Витамины для собак крупных пород 8in1 Excel Brewer's Yeast for large breed 80 шт</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Витамины для собак Glucosamine для суставов 55 таблеток</t>
+          <t>Витамины для собак для суставов 8in1 Excel Glucosamine 55 шт</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Витамины для собак Glucosamine для суставов 55 таблеток</t>
+          <t>Витамины для собак для суставов 8in1 Excel Glucosamine 55 шт</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Витамины для собак Glucosamine для суставов 55 таблеток</t>
+          <t>Витамины для собак для суставов 8in1 Excel Glucosamine 55 шт</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Витамины для собак Glucosamine для суставов 55 таблеток</t>
+          <t>Витамины для собак для суставов 8in1 Excel Glucosamine 55 шт</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Витамины для собак мелких пород 70 таблеток</t>
+          <t>Витамины для собак мелких пород Excel Multi Vitamin Small Breed 70 шт</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Витамины для собак мелких пород 70 таблеток</t>
+          <t>Витамины для собак мелких пород Excel Multi Vitamin Small Breed 70 шт</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Витамины для собак мелких пород 70 таблеток</t>
+          <t>Витамины для собак мелких пород Excel Multi Vitamin Small Breed 70 шт</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Витамины для собак мелких пород 70 таблеток</t>
+          <t>Витамины для собак мелких пород Excel Multi Vitamin Small Breed 70 шт</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Витамины для собак мелких пород 70 таблеток</t>
+          <t>Витамины для собак мелких пород Excel Multi Vitamin Small Breed 70 шт</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Витамины для пожилых собак от 5 лет 70 таблеток</t>
+          <t>Витамины для пожилых собак от 5 лет 8in1 Excel Multi Vitamin Senior 70 шт</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Витамины для пожилых собак от 5 лет 70 таблеток</t>
+          <t>Витамины для пожилых собак от 5 лет 8in1 Excel Multi Vitamin Senior 70 шт</t>
         </is>
       </c>
       <c r="C19" t="n">

</xml_diff>

<commit_message>
update ozon ff boxes 2026-08-19
</commit_message>
<xml_diff>
--- a/supplies/108441550-1.xlsx
+++ b/supplies/108441550-1.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Инфо" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ПО КОРОБАМ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ПО ТОВАРУ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инфо" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ПО КОРОБАМ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ПО ТОВАРУ" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>